<commit_message>
Initial commit with proper .gitignore setup
</commit_message>
<xml_diff>
--- a/frontend/public/cashroom-template.xlsx
+++ b/frontend/public/cashroom-template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tarandeeps\Downloads\compass_complete-main (1)\compass_complete-main\frontend\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\Backup\Compass-Cashroom-V11\frontend\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B36ABE59-B44B-44F6-A38F-C6E65CAC8137}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{905D4DEA-D22A-4ECE-BA4B-538EA3B51DB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -409,7 +409,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="28">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -636,9 +636,39 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom style="thin">
         <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="8"/>
       </bottom>
       <diagonal/>
     </border>
@@ -751,7 +781,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
@@ -792,37 +822,39 @@
     <xf numFmtId="39" fontId="1" fillId="4" borderId="18" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="39" fontId="1" fillId="3" borderId="19" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="39" fontId="1" fillId="4" borderId="19" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="39" fontId="1" fillId="3" borderId="20" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="39" fontId="1" fillId="4" borderId="21" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="39" fontId="1" fillId="2" borderId="22" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="39" fontId="6" fillId="3" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="39" fontId="1" fillId="2" borderId="20" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="39" fontId="6" fillId="3" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="39" fontId="1" fillId="2" borderId="19" xfId="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="23" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="24" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="26" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="39" fontId="1" fillId="4" borderId="25" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="39" fontId="1" fillId="4" borderId="27" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="26" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="28" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="39" fontId="1" fillId="3" borderId="16" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="22" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="23" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="27" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="24" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="25" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="29" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="13" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="39" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="22" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="23" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="24" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="25" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="39" fontId="1" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="29" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1251,11 +1283,11 @@
       <c r="A4" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="B4" s="73" t="s">
+      <c r="B4" s="75" t="s">
         <v>84</v>
       </c>
-      <c r="C4" s="73"/>
-      <c r="D4" s="73"/>
+      <c r="C4" s="75"/>
+      <c r="D4" s="75"/>
       <c r="E4" s="2"/>
       <c r="F4" s="4"/>
       <c r="G4" s="8" t="s">
@@ -1306,14 +1338,14 @@
       <c r="A7" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="35">
+      <c r="B7" s="38">
         <v>0</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="E7" s="35">
+      <c r="E7" s="40">
         <v>0</v>
       </c>
       <c r="G7" s="23"/>
@@ -1333,7 +1365,9 @@
       <c r="A8" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="34"/>
+      <c r="B8" s="34">
+        <v>0</v>
+      </c>
       <c r="C8" s="2"/>
       <c r="D8" s="26" t="s">
         <v>15</v>
@@ -1345,7 +1379,7 @@
         <v>13</v>
       </c>
       <c r="H8" s="14"/>
-      <c r="I8" s="35">
+      <c r="I8" s="14">
         <v>0</v>
       </c>
       <c r="J8" s="28">
@@ -1364,7 +1398,7 @@
       <c r="A9" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="35">
+      <c r="B9" s="34">
         <v>0</v>
       </c>
       <c r="C9" s="2"/>
@@ -1378,7 +1412,7 @@
         <v>15</v>
       </c>
       <c r="H9" s="14"/>
-      <c r="I9" s="35">
+      <c r="I9" s="14">
         <v>0</v>
       </c>
       <c r="J9" s="28">
@@ -1397,7 +1431,7 @@
       <c r="A10" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="35">
+      <c r="B10" s="34">
         <v>0</v>
       </c>
       <c r="C10" s="2"/>
@@ -1411,7 +1445,7 @@
         <v>17</v>
       </c>
       <c r="H10" s="14"/>
-      <c r="I10" s="35">
+      <c r="I10" s="14">
         <v>0</v>
       </c>
       <c r="J10" s="28">
@@ -1430,7 +1464,7 @@
       <c r="A11" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="35">
+      <c r="B11" s="34">
         <v>0</v>
       </c>
       <c r="C11" s="2"/>
@@ -1444,7 +1478,7 @@
         <v>19</v>
       </c>
       <c r="H11" s="14"/>
-      <c r="I11" s="35">
+      <c r="I11" s="14">
         <v>0</v>
       </c>
       <c r="J11" s="28">
@@ -1493,12 +1527,12 @@
       <c r="B13" s="34"/>
       <c r="C13" s="2"/>
       <c r="D13" s="30"/>
-      <c r="E13" s="39"/>
+      <c r="E13" s="41"/>
       <c r="G13" s="26" t="s">
         <v>22</v>
       </c>
       <c r="H13" s="14"/>
-      <c r="I13" s="35">
+      <c r="I13" s="14">
         <v>0</v>
       </c>
       <c r="J13" s="28">
@@ -1517,21 +1551,21 @@
       <c r="A14" s="30" t="s">
         <v>76</v>
       </c>
-      <c r="B14" s="41"/>
+      <c r="B14" s="43"/>
       <c r="C14" s="2"/>
       <c r="D14" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="E14" s="38">
+      <c r="E14" s="39">
         <f>SUM(E7:E12)</f>
         <v>0</v>
       </c>
-      <c r="G14" s="42"/>
-      <c r="H14" s="43"/>
-      <c r="I14" s="35">
-        <v>0</v>
-      </c>
-      <c r="J14" s="44">
+      <c r="G14" s="44"/>
+      <c r="H14" s="45"/>
+      <c r="I14" s="45">
+        <v>0</v>
+      </c>
+      <c r="J14" s="46">
         <v>0.01</v>
       </c>
       <c r="K14" s="15">
@@ -1547,7 +1581,7 @@
       <c r="A15" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="40">
+      <c r="B15" s="42">
         <f>SUM(B7:B14)</f>
         <v>0</v>
       </c>
@@ -1560,7 +1594,7 @@
       <c r="K15" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="L15" s="40">
+      <c r="L15" s="42">
         <f>SUM(L8:L14)</f>
         <v>0</v>
       </c>
@@ -1569,15 +1603,15 @@
       <c r="A17" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="B17" s="51"/>
-      <c r="C17" s="52"/>
+      <c r="B17" s="53"/>
+      <c r="C17" s="54"/>
       <c r="E17" s="36" t="s">
         <v>51</v>
       </c>
-      <c r="F17" s="51"/>
-      <c r="G17" s="51"/>
-      <c r="H17" s="51"/>
-      <c r="I17" s="51"/>
+      <c r="F17" s="53"/>
+      <c r="G17" s="53"/>
+      <c r="H17" s="53"/>
+      <c r="I17" s="53"/>
       <c r="J17" s="11"/>
       <c r="K17" s="11"/>
       <c r="L17" s="12"/>
@@ -1624,13 +1658,13 @@
       <c r="C19" s="35">
         <v>0</v>
       </c>
-      <c r="E19" s="48">
-        <v>3</v>
-      </c>
-      <c r="F19" s="49" t="s">
+      <c r="E19" s="50">
+        <v>0</v>
+      </c>
+      <c r="F19" s="51" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="35">
+      <c r="G19" s="18">
         <v>0</v>
       </c>
       <c r="H19" s="19">
@@ -1638,7 +1672,7 @@
         <v>0</v>
       </c>
       <c r="I19" s="20"/>
-      <c r="J19" s="49" t="s">
+      <c r="J19" s="51" t="s">
         <v>29</v>
       </c>
       <c r="K19" s="18"/>
@@ -1658,13 +1692,13 @@
       <c r="C20" s="35">
         <v>0</v>
       </c>
-      <c r="E20" s="48">
-        <v>5</v>
-      </c>
-      <c r="F20" s="49" t="s">
+      <c r="E20" s="50">
+        <v>0</v>
+      </c>
+      <c r="F20" s="51" t="s">
         <v>29</v>
       </c>
-      <c r="G20" s="35">
+      <c r="G20" s="18">
         <v>0</v>
       </c>
       <c r="H20" s="19">
@@ -1672,7 +1706,7 @@
         <v>0</v>
       </c>
       <c r="I20" s="20"/>
-      <c r="J20" s="49" t="s">
+      <c r="J20" s="51" t="s">
         <v>29</v>
       </c>
       <c r="K20" s="18"/>
@@ -1692,13 +1726,13 @@
       <c r="C21" s="35">
         <v>0</v>
       </c>
-      <c r="E21" s="48">
-        <v>1</v>
-      </c>
-      <c r="F21" s="49" t="s">
+      <c r="E21" s="50">
+        <v>0</v>
+      </c>
+      <c r="F21" s="51" t="s">
         <v>29</v>
       </c>
-      <c r="G21" s="35">
+      <c r="G21" s="18">
         <v>0</v>
       </c>
       <c r="H21" s="19">
@@ -1706,7 +1740,7 @@
         <v>0</v>
       </c>
       <c r="I21" s="20"/>
-      <c r="J21" s="49" t="s">
+      <c r="J21" s="51" t="s">
         <v>29</v>
       </c>
       <c r="K21" s="18"/>
@@ -1726,8 +1760,8 @@
       <c r="C22" s="35">
         <v>0</v>
       </c>
-      <c r="E22" s="48"/>
-      <c r="F22" s="49" t="s">
+      <c r="E22" s="50"/>
+      <c r="F22" s="51" t="s">
         <v>29</v>
       </c>
       <c r="G22" s="18"/>
@@ -1736,7 +1770,7 @@
         <v>0</v>
       </c>
       <c r="I22" s="20"/>
-      <c r="J22" s="49" t="s">
+      <c r="J22" s="51" t="s">
         <v>29</v>
       </c>
       <c r="K22" s="18"/>
@@ -1748,13 +1782,13 @@
     </row>
     <row r="23" spans="1:13" ht="15.5">
       <c r="A23" s="26"/>
-      <c r="B23" s="45"/>
-      <c r="C23" s="50"/>
-      <c r="E23" s="48"/>
-      <c r="F23" s="49" t="s">
+      <c r="B23" s="47"/>
+      <c r="C23" s="52"/>
+      <c r="E23" s="50"/>
+      <c r="F23" s="51" t="s">
         <v>29</v>
       </c>
-      <c r="G23" s="35">
+      <c r="G23" s="18">
         <v>0</v>
       </c>
       <c r="H23" s="19">
@@ -1762,7 +1796,7 @@
         <v>0</v>
       </c>
       <c r="I23" s="20"/>
-      <c r="J23" s="49" t="s">
+      <c r="J23" s="51" t="s">
         <v>29</v>
       </c>
       <c r="K23" s="18"/>
@@ -1773,8 +1807,8 @@
       <c r="M23" s="2"/>
     </row>
     <row r="24" spans="1:13" ht="15.5">
-      <c r="A24" s="46"/>
-      <c r="B24" s="47" t="s">
+      <c r="A24" s="48"/>
+      <c r="B24" s="49" t="s">
         <v>31</v>
       </c>
       <c r="C24" s="17">
@@ -1784,7 +1818,7 @@
       <c r="E24" s="26"/>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
-      <c r="H24" s="49"/>
+      <c r="H24" s="51"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
@@ -1792,13 +1826,13 @@
       <c r="M24" s="2"/>
     </row>
     <row r="25" spans="1:13" ht="15.5">
-      <c r="E25" s="46"/>
-      <c r="F25" s="47"/>
-      <c r="G25" s="47"/>
-      <c r="H25" s="56"/>
-      <c r="I25" s="47"/>
-      <c r="J25" s="47"/>
-      <c r="K25" s="57" t="s">
+      <c r="E25" s="48"/>
+      <c r="F25" s="49"/>
+      <c r="G25" s="49"/>
+      <c r="H25" s="58"/>
+      <c r="I25" s="49"/>
+      <c r="J25" s="49"/>
+      <c r="K25" s="59" t="s">
         <v>52</v>
       </c>
       <c r="L25" s="17">
@@ -1814,9 +1848,9 @@
       <c r="A27" s="36" t="s">
         <v>32</v>
       </c>
-      <c r="B27" s="51"/>
-      <c r="C27" s="51"/>
-      <c r="D27" s="51"/>
+      <c r="B27" s="53"/>
+      <c r="C27" s="53"/>
+      <c r="D27" s="53"/>
       <c r="E27" s="12"/>
       <c r="M27" s="2"/>
     </row>
@@ -1837,8 +1871,8 @@
       <c r="M28" s="2"/>
     </row>
     <row r="29" spans="1:13" ht="15.5">
-      <c r="A29" s="48"/>
-      <c r="B29" s="49" t="s">
+      <c r="A29" s="50"/>
+      <c r="B29" s="51" t="s">
         <v>29</v>
       </c>
       <c r="C29" s="14"/>
@@ -1850,8 +1884,8 @@
       <c r="M29" s="2"/>
     </row>
     <row r="30" spans="1:13" ht="15.5">
-      <c r="A30" s="48"/>
-      <c r="B30" s="49" t="s">
+      <c r="A30" s="50"/>
+      <c r="B30" s="51" t="s">
         <v>29</v>
       </c>
       <c r="C30" s="14"/>
@@ -1863,8 +1897,8 @@
       <c r="F30" s="2"/>
     </row>
     <row r="31" spans="1:13" ht="15.5">
-      <c r="A31" s="48"/>
-      <c r="B31" s="49" t="s">
+      <c r="A31" s="50"/>
+      <c r="B31" s="51" t="s">
         <v>29</v>
       </c>
       <c r="C31" s="14"/>
@@ -1876,25 +1910,25 @@
       <c r="F31" s="2"/>
     </row>
     <row r="32" spans="1:13" ht="15.5">
-      <c r="A32" s="53"/>
-      <c r="B32" s="49" t="s">
+      <c r="A32" s="55"/>
+      <c r="B32" s="51" t="s">
         <v>29</v>
       </c>
-      <c r="C32" s="45"/>
+      <c r="C32" s="47"/>
       <c r="D32" s="2"/>
-      <c r="E32" s="54">
+      <c r="E32" s="56">
         <f>A32*C32</f>
         <v>0</v>
       </c>
       <c r="F32" s="2"/>
     </row>
     <row r="33" spans="1:15" ht="15.5">
-      <c r="A33" s="55"/>
-      <c r="B33" s="56"/>
-      <c r="C33" s="56" t="s">
+      <c r="A33" s="57"/>
+      <c r="B33" s="58"/>
+      <c r="C33" s="58" t="s">
         <v>35</v>
       </c>
-      <c r="D33" s="47"/>
+      <c r="D33" s="49"/>
       <c r="E33" s="19">
         <f>SUM(E29:E32)</f>
         <v>0</v>
@@ -1908,29 +1942,29 @@
       <c r="F35" s="2"/>
     </row>
     <row r="36" spans="1:15" ht="15.5">
-      <c r="A36" s="63" t="s">
+      <c r="A36" s="65" t="s">
         <v>77</v>
       </c>
-      <c r="B36" s="56"/>
-      <c r="C36" s="56"/>
-      <c r="D36" s="47"/>
-      <c r="E36" s="57"/>
+      <c r="B36" s="58"/>
+      <c r="C36" s="58"/>
+      <c r="D36" s="49"/>
+      <c r="E36" s="59"/>
       <c r="F36" s="2"/>
     </row>
     <row r="37" spans="1:15" ht="15.5">
-      <c r="A37" s="58"/>
-      <c r="B37" s="59"/>
-      <c r="C37" s="59"/>
+      <c r="A37" s="60"/>
+      <c r="B37" s="61"/>
+      <c r="C37" s="61"/>
       <c r="D37" s="24"/>
       <c r="E37" s="25"/>
       <c r="F37" s="2"/>
     </row>
     <row r="38" spans="1:15" ht="15.5">
-      <c r="A38" s="60" t="s">
+      <c r="A38" s="62" t="s">
         <v>36</v>
       </c>
       <c r="B38" s="13"/>
-      <c r="C38" s="49"/>
+      <c r="C38" s="51"/>
       <c r="D38" s="2"/>
       <c r="E38" s="27"/>
       <c r="F38" s="2"/>
@@ -1938,32 +1972,32 @@
       <c r="L38" s="2"/>
     </row>
     <row r="39" spans="1:15" ht="15.5">
-      <c r="A39" s="60" t="s">
+      <c r="A39" s="62" t="s">
         <v>37</v>
       </c>
       <c r="B39" s="13"/>
-      <c r="C39" s="49"/>
+      <c r="C39" s="51"/>
       <c r="D39" s="2"/>
       <c r="E39" s="27"/>
       <c r="F39" s="2"/>
       <c r="G39" s="8"/>
-      <c r="H39" s="72" t="s">
+      <c r="H39" s="74" t="s">
         <v>41</v>
       </c>
-      <c r="I39" s="72"/>
-      <c r="J39" s="72"/>
+      <c r="I39" s="74"/>
+      <c r="J39" s="74"/>
       <c r="K39" s="8"/>
       <c r="L39" s="8"/>
       <c r="M39" s="2"/>
     </row>
     <row r="40" spans="1:15" ht="15.5">
       <c r="A40" s="26"/>
-      <c r="B40" s="61"/>
+      <c r="B40" s="63"/>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
       <c r="E40" s="27"/>
       <c r="F40" s="2"/>
-      <c r="G40" s="70" t="s">
+      <c r="G40" s="72" t="s">
         <v>53</v>
       </c>
       <c r="H40" s="2" t="s">
@@ -1984,9 +2018,9 @@
       <c r="B41" s="19"/>
       <c r="C41" s="7"/>
       <c r="D41" s="7"/>
-      <c r="E41" s="62"/>
+      <c r="E41" s="64"/>
       <c r="F41" s="2"/>
-      <c r="G41" s="70" t="s">
+      <c r="G41" s="72" t="s">
         <v>54</v>
       </c>
       <c r="H41" s="2" t="s">
@@ -2006,7 +2040,7 @@
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
       <c r="F42" s="2"/>
-      <c r="G42" s="70" t="s">
+      <c r="G42" s="72" t="s">
         <v>55</v>
       </c>
       <c r="H42" s="2" t="s">
@@ -2020,15 +2054,15 @@
       </c>
     </row>
     <row r="43" spans="1:15" ht="15.5">
-      <c r="A43" s="64" t="s">
+      <c r="A43" s="66" t="s">
         <v>39</v>
       </c>
-      <c r="B43" s="65"/>
-      <c r="C43" s="65"/>
-      <c r="D43" s="47"/>
-      <c r="E43" s="57"/>
+      <c r="B43" s="67"/>
+      <c r="C43" s="67"/>
+      <c r="D43" s="49"/>
+      <c r="E43" s="59"/>
       <c r="F43" s="2"/>
-      <c r="G43" s="70" t="s">
+      <c r="G43" s="72" t="s">
         <v>56</v>
       </c>
       <c r="H43" s="2" t="s">
@@ -2050,7 +2084,7 @@
       <c r="D44" s="2"/>
       <c r="E44" s="27"/>
       <c r="F44" s="2"/>
-      <c r="G44" s="70" t="s">
+      <c r="G44" s="72" t="s">
         <v>57</v>
       </c>
       <c r="H44" s="2" t="s">
@@ -2072,7 +2106,7 @@
       <c r="D45" s="2"/>
       <c r="E45" s="27"/>
       <c r="F45" s="2"/>
-      <c r="G45" s="70" t="s">
+      <c r="G45" s="72" t="s">
         <v>58</v>
       </c>
       <c r="H45" s="2" t="s">
@@ -2092,10 +2126,10 @@
       <c r="D46" s="2"/>
       <c r="E46" s="27"/>
       <c r="F46" s="2"/>
-      <c r="G46" s="70" t="s">
+      <c r="G46" s="72" t="s">
         <v>64</v>
       </c>
-      <c r="H46" s="69" t="s">
+      <c r="H46" s="71" t="s">
         <v>78</v>
       </c>
       <c r="I46" s="2"/>
@@ -2109,14 +2143,14 @@
       <c r="A47" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="B47" s="74">
+      <c r="B47" s="76">
         <v>0</v>
       </c>
       <c r="C47" s="7"/>
       <c r="D47" s="7"/>
-      <c r="E47" s="62"/>
+      <c r="E47" s="64"/>
       <c r="F47" s="2"/>
-      <c r="G47" s="70"/>
+      <c r="G47" s="72"/>
       <c r="H47" s="2" t="s">
         <v>65</v>
       </c>
@@ -2132,7 +2166,7 @@
       <c r="D48" s="2"/>
       <c r="E48" s="2"/>
       <c r="F48" s="2"/>
-      <c r="G48" s="70"/>
+      <c r="G48" s="72"/>
       <c r="H48" s="2" t="s">
         <v>45</v>
       </c>
@@ -2151,7 +2185,7 @@
       <c r="D49" s="2"/>
       <c r="E49" s="2"/>
       <c r="F49" s="2"/>
-      <c r="G49" s="70" t="s">
+      <c r="G49" s="72" t="s">
         <v>74</v>
       </c>
       <c r="H49" s="2" t="s">
@@ -2166,18 +2200,18 @@
       <c r="O49" s="2"/>
     </row>
     <row r="50" spans="1:15" ht="15.5">
-      <c r="A50" s="64" t="s">
+      <c r="A50" s="66" t="s">
         <v>44</v>
       </c>
-      <c r="B50" s="65"/>
-      <c r="C50" s="65"/>
-      <c r="D50" s="65"/>
-      <c r="E50" s="67"/>
+      <c r="B50" s="67"/>
+      <c r="C50" s="67"/>
+      <c r="D50" s="67"/>
+      <c r="E50" s="69"/>
       <c r="F50" s="2"/>
-      <c r="G50" s="71" t="s">
+      <c r="G50" s="73" t="s">
         <v>73</v>
       </c>
-      <c r="H50" s="69" t="s">
+      <c r="H50" s="71" t="s">
         <v>81</v>
       </c>
       <c r="L50" s="21">
@@ -2193,11 +2227,11 @@
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
-      <c r="E51" s="35">
+      <c r="E51" s="13">
         <v>0</v>
       </c>
       <c r="F51" s="2"/>
-      <c r="G51" s="70" t="s">
+      <c r="G51" s="72" t="s">
         <v>67</v>
       </c>
       <c r="H51" s="2" t="s">
@@ -2216,7 +2250,7 @@
       <c r="D52" s="2"/>
       <c r="E52" s="27"/>
       <c r="F52" s="2"/>
-      <c r="G52" s="70" t="s">
+      <c r="G52" s="72" t="s">
         <v>69</v>
       </c>
       <c r="H52" s="2" t="s">
@@ -2234,14 +2268,14 @@
       <c r="A53" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="B53" s="66"/>
+      <c r="B53" s="68"/>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
       <c r="E53" s="13">
         <v>0</v>
       </c>
       <c r="F53" s="2"/>
-      <c r="G53" s="69"/>
+      <c r="G53" s="71"/>
       <c r="H53" s="2" t="s">
         <v>71</v>
       </c>
@@ -2258,7 +2292,7 @@
       <c r="D54" s="2"/>
       <c r="E54" s="27"/>
       <c r="F54" s="2"/>
-      <c r="G54" s="69"/>
+      <c r="G54" s="71"/>
       <c r="H54" s="2" t="s">
         <v>47</v>
       </c>
@@ -2272,12 +2306,12 @@
     </row>
     <row r="55" spans="1:15" ht="15.5">
       <c r="A55" s="26"/>
-      <c r="B55" s="61"/>
+      <c r="B55" s="63"/>
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
       <c r="E55" s="27"/>
       <c r="F55" s="2"/>
-      <c r="G55" s="69"/>
+      <c r="G55" s="71"/>
       <c r="H55" s="2" t="s">
         <v>72</v>
       </c>
@@ -2289,12 +2323,12 @@
       <c r="O55" s="2"/>
     </row>
     <row r="56" spans="1:15" ht="15.5">
-      <c r="A56" s="46" t="s">
+      <c r="A56" s="48" t="s">
         <v>46</v>
       </c>
-      <c r="B56" s="68"/>
-      <c r="C56" s="47"/>
-      <c r="D56" s="57"/>
+      <c r="B56" s="70"/>
+      <c r="C56" s="49"/>
+      <c r="D56" s="59"/>
       <c r="E56" s="19">
         <f>E51+E53</f>
         <v>0</v>
@@ -2451,6 +2485,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F1CDF4AE13F64D40BBB65824B29FAA7E" ma:contentTypeVersion="8" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0d2301f73a884384ddd5c8a4d00c99b5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="165b96c2-f4bb-42d4-bd0e-5bd22b3c2c99" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f44d8ff651ee59b55465c93f60004624" ns2:_="">
     <xsd:import namespace="165b96c2-f4bb-42d4-bd0e-5bd22b3c2c99"/>
@@ -2618,22 +2667,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B24100DD-9604-4D6D-B080-152095F3FAE0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="165b96c2-f4bb-42d4-bd0e-5bd22b3c2c99"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1677FD12-FF7E-4FED-B391-03DF70F45953}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC46D7E8-5F30-4E91-A1E5-4030A3C193DF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2651,30 +2709,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1677FD12-FF7E-4FED-B391-03DF70F45953}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B24100DD-9604-4D6D-B080-152095F3FAE0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="165b96c2-f4bb-42d4-bd0e-5bd22b3c2c99"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{cd62b7dd-4b48-44bd-90e7-e143a22c8ead}" enabled="0" method="" siteId="{cd62b7dd-4b48-44bd-90e7-e143a22c8ead}" removed="1"/>

</xml_diff>

<commit_message>
fix: Replace operator sample Excel with correct Cashroom Count Worksheet
Added e2e test that downloads sample Excel and re-uploads it
to verify no parsing errors.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/cashroom-template.xlsx
+++ b/frontend/public/cashroom-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\Backup\Compass-Cashroom-V11\frontend\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pankhurig\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{905D4DEA-D22A-4ECE-BA4B-538EA3B51DB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81F3B719-CA37-424D-ABF3-60AA1624D9E7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="19416" windowHeight="10416" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1-20-26" sheetId="12" r:id="rId1"/>
@@ -23,23 +23,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="85">
   <si>
     <t>Canteen Vending Services</t>
   </si>
@@ -243,9 +232,6 @@
   </si>
   <si>
     <t>J</t>
-  </si>
-  <si>
-    <t>Replenishment in Transit</t>
   </si>
   <si>
     <t>K</t>
@@ -409,7 +395,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="30">
+  <borders count="28">
     <border>
       <left/>
       <right/>
@@ -636,39 +622,9 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
       <top/>
       <bottom style="thin">
         <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="8"/>
       </bottom>
       <diagonal/>
     </border>
@@ -781,7 +737,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
@@ -822,39 +778,37 @@
     <xf numFmtId="39" fontId="1" fillId="4" borderId="18" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="39" fontId="1" fillId="4" borderId="19" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="39" fontId="1" fillId="3" borderId="20" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="39" fontId="1" fillId="4" borderId="21" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="39" fontId="1" fillId="2" borderId="22" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="39" fontId="6" fillId="3" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="39" fontId="1" fillId="3" borderId="19" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="39" fontId="1" fillId="2" borderId="20" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="39" fontId="6" fillId="3" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="39" fontId="1" fillId="2" borderId="19" xfId="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="23" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="26" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="24" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="39" fontId="1" fillId="4" borderId="27" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="39" fontId="1" fillId="4" borderId="25" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="28" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="26" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="39" fontId="1" fillId="3" borderId="16" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="24" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="25" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="29" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="22" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="23" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="27" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="13" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="39" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="24" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="25" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="22" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="23" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="39" fontId="1" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="29" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1204,23 +1158,22 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:O68"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="14.453125" customWidth="1"/>
-    <col min="2" max="2" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.26953125" customWidth="1"/>
-    <col min="5" max="5" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.1796875" customWidth="1"/>
-    <col min="8" max="8" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.54296875" customWidth="1"/>
-    <col min="12" max="12" width="11.453125" customWidth="1"/>
-    <col min="13" max="13" width="11.26953125" customWidth="1"/>
-    <col min="14" max="14" width="11.7265625" customWidth="1"/>
-    <col min="16" max="16" width="10.26953125" customWidth="1"/>
+    <col min="1" max="1" width="14.5" customWidth="1"/>
+    <col min="2" max="2" width="12.69921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.296875" customWidth="1"/>
+    <col min="5" max="5" width="10.796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.19921875" customWidth="1"/>
+    <col min="8" max="8" width="10.796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="11.5" customWidth="1"/>
+    <col min="13" max="13" width="11.296875" customWidth="1"/>
+    <col min="14" max="14" width="11.69921875" customWidth="1"/>
+    <col min="16" max="16" width="10.296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.5">
+    <row r="1" spans="1:13" ht="15.6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1239,7 +1192,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="20">
+    <row r="2" spans="1:13" ht="21">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1260,7 +1213,7 @@
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
     </row>
-    <row r="3" spans="1:13" ht="20">
+    <row r="3" spans="1:13" ht="21">
       <c r="A3" s="8" t="s">
         <v>5</v>
       </c>
@@ -1279,19 +1232,19 @@
       <c r="L3" s="2"/>
       <c r="M3" s="2"/>
     </row>
-    <row r="4" spans="1:13" ht="20">
+    <row r="4" spans="1:13" ht="21">
       <c r="A4" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="B4" s="75" t="s">
-        <v>84</v>
-      </c>
-      <c r="C4" s="75"/>
-      <c r="D4" s="75"/>
+        <v>81</v>
+      </c>
+      <c r="B4" s="73" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4" s="73"/>
+      <c r="D4" s="73"/>
       <c r="E4" s="2"/>
       <c r="F4" s="4"/>
       <c r="G4" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H4" s="10"/>
       <c r="I4" s="8"/>
@@ -1300,7 +1253,7 @@
       <c r="L4" s="8"/>
       <c r="M4" s="2"/>
     </row>
-    <row r="5" spans="1:13" ht="15.5">
+    <row r="5" spans="1:13" ht="15">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -1315,7 +1268,7 @@
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
     </row>
-    <row r="6" spans="1:13" ht="15.5">
+    <row r="6" spans="1:13" ht="15.6">
       <c r="A6" s="36" t="s">
         <v>6</v>
       </c>
@@ -1326,7 +1279,7 @@
       </c>
       <c r="E6" s="25"/>
       <c r="G6" s="37" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H6" s="24"/>
       <c r="I6" s="24"/>
@@ -1334,19 +1287,19 @@
       <c r="K6" s="24"/>
       <c r="L6" s="25"/>
     </row>
-    <row r="7" spans="1:13" ht="15.5">
+    <row r="7" spans="1:13" ht="15">
       <c r="A7" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="38">
-        <v>0</v>
+      <c r="B7" s="35">
+        <v>1000</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="E7" s="40">
-        <v>0</v>
+      <c r="E7" s="35">
+        <v>200</v>
       </c>
       <c r="G7" s="23"/>
       <c r="H7" s="24" t="s">
@@ -1361,25 +1314,27 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="15.5">
+    <row r="8" spans="1:13" ht="15">
       <c r="A8" s="26" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="34">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="26" t="s">
         <v>15</v>
       </c>
       <c r="E8" s="35">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G8" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14">
+      <c r="H8" s="14">
+        <v>100</v>
+      </c>
+      <c r="I8" s="35">
         <v>0</v>
       </c>
       <c r="J8" s="28">
@@ -1387,19 +1342,19 @@
       </c>
       <c r="K8" s="15">
         <f t="shared" ref="K8:K14" si="0">+H8+I8</f>
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="L8" s="16">
-        <f t="shared" ref="L8:L14" si="1">+K8*J8</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" ht="15.5">
+        <f t="shared" ref="L8:L11" si="1">+K8*J8</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="15">
       <c r="A9" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="34">
-        <v>0</v>
+      <c r="B9" s="35">
+        <v>60</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="26" t="s">
@@ -1412,7 +1367,7 @@
         <v>15</v>
       </c>
       <c r="H9" s="14"/>
-      <c r="I9" s="14">
+      <c r="I9" s="35">
         <v>0</v>
       </c>
       <c r="J9" s="28">
@@ -1427,12 +1382,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="15.5">
+    <row r="10" spans="1:13" ht="15">
       <c r="A10" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="34">
-        <v>0</v>
+      <c r="B10" s="35">
+        <v>150</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="26" t="s">
@@ -1445,7 +1400,7 @@
         <v>17</v>
       </c>
       <c r="H10" s="14"/>
-      <c r="I10" s="14">
+      <c r="I10" s="35">
         <v>0</v>
       </c>
       <c r="J10" s="28">
@@ -1460,25 +1415,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="15.5">
+    <row r="11" spans="1:13" ht="15">
       <c r="A11" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="34">
-        <v>0</v>
+      <c r="B11" s="35">
+        <v>100</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="26" t="s">
         <v>21</v>
       </c>
       <c r="E11" s="35">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="G11" s="26" t="s">
         <v>19</v>
       </c>
       <c r="H11" s="14"/>
-      <c r="I11" s="14">
+      <c r="I11" s="35">
         <v>0</v>
       </c>
       <c r="J11" s="28">
@@ -1493,97 +1448,104 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="15.5">
+    <row r="12" spans="1:13" ht="15">
       <c r="A12" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="34"/>
+      <c r="B12" s="34">
+        <v>200</v>
+      </c>
       <c r="C12" s="2"/>
       <c r="D12" s="26" t="s">
         <v>22</v>
       </c>
       <c r="E12" s="35">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G12" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="H12" s="14"/>
+      <c r="H12" s="14">
+        <v>200</v>
+      </c>
       <c r="I12" s="14"/>
-      <c r="J12" s="28"/>
+      <c r="J12" s="28">
+        <v>0.05</v>
+      </c>
       <c r="K12" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>+H12+I12</f>
+        <v>200</v>
       </c>
       <c r="L12" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" ht="15.5">
+        <f>+K12*J12</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="15">
       <c r="A13" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="34"/>
+      <c r="B13" s="34">
+        <v>400</v>
+      </c>
       <c r="C13" s="2"/>
       <c r="D13" s="30"/>
-      <c r="E13" s="41"/>
+      <c r="E13" s="39"/>
       <c r="G13" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="H13" s="14"/>
-      <c r="I13" s="14">
-        <v>0</v>
-      </c>
-      <c r="J13" s="28">
-        <v>0.05</v>
+      <c r="H13" s="14">
+        <v>100</v>
+      </c>
+      <c r="I13" s="35">
+        <v>0</v>
+      </c>
+      <c r="J13" s="44">
+        <v>0.01</v>
       </c>
       <c r="K13" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="L13" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" ht="15.5">
+        <f>+K13*J12</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="15">
       <c r="A14" s="30" t="s">
-        <v>76</v>
-      </c>
-      <c r="B14" s="43"/>
+        <v>75</v>
+      </c>
+      <c r="B14" s="41"/>
       <c r="C14" s="2"/>
       <c r="D14" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="E14" s="39">
+      <c r="E14" s="38">
         <f>SUM(E7:E12)</f>
-        <v>0</v>
-      </c>
-      <c r="G14" s="44"/>
-      <c r="H14" s="45"/>
-      <c r="I14" s="45">
-        <v>0</v>
-      </c>
-      <c r="J14" s="46">
-        <v>0.01</v>
+        <v>722</v>
+      </c>
+      <c r="G14" s="42"/>
+      <c r="H14" s="43"/>
+      <c r="I14" s="35">
+        <v>0</v>
       </c>
       <c r="K14" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L14" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" ht="15.5">
+        <f>+K14*J13</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="15">
       <c r="A15" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="42">
+      <c r="B15" s="40">
         <f>SUM(B7:B14)</f>
-        <v>0</v>
+        <v>1933</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
@@ -1594,29 +1556,29 @@
       <c r="K15" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="L15" s="42">
+      <c r="L15" s="40">
         <f>SUM(L8:L14)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" ht="15.5">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="15.6">
       <c r="A17" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="B17" s="53"/>
-      <c r="C17" s="54"/>
+      <c r="B17" s="51"/>
+      <c r="C17" s="52"/>
       <c r="E17" s="36" t="s">
         <v>51</v>
       </c>
-      <c r="F17" s="53"/>
-      <c r="G17" s="53"/>
-      <c r="H17" s="53"/>
-      <c r="I17" s="53"/>
+      <c r="F17" s="51"/>
+      <c r="G17" s="51"/>
+      <c r="H17" s="51"/>
+      <c r="I17" s="51"/>
       <c r="J17" s="11"/>
       <c r="K17" s="11"/>
       <c r="L17" s="12"/>
     </row>
-    <row r="18" spans="1:13" ht="15.5">
+    <row r="18" spans="1:13" ht="15">
       <c r="A18" s="23" t="s">
         <v>24</v>
       </c>
@@ -1648,31 +1610,31 @@
       </c>
       <c r="M18" s="2"/>
     </row>
-    <row r="19" spans="1:13" ht="15.5">
+    <row r="19" spans="1:13" ht="15">
       <c r="A19" s="26" t="s">
         <v>13</v>
       </c>
       <c r="B19" s="14">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C19" s="35">
         <v>0</v>
       </c>
-      <c r="E19" s="50">
-        <v>0</v>
-      </c>
-      <c r="F19" s="51" t="s">
+      <c r="E19" s="48">
+        <v>3</v>
+      </c>
+      <c r="F19" s="49" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="18">
-        <v>0</v>
+      <c r="G19" s="35">
+        <v>400</v>
       </c>
       <c r="H19" s="19">
         <f>E19*G19</f>
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I19" s="20"/>
-      <c r="J19" s="51" t="s">
+      <c r="J19" s="49" t="s">
         <v>29</v>
       </c>
       <c r="K19" s="18"/>
@@ -1682,31 +1644,31 @@
       </c>
       <c r="M19" s="2"/>
     </row>
-    <row r="20" spans="1:13" ht="15.5">
+    <row r="20" spans="1:13" ht="15">
       <c r="A20" s="26" t="s">
         <v>17</v>
       </c>
       <c r="B20" s="14">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C20" s="35">
         <v>0</v>
       </c>
-      <c r="E20" s="50">
-        <v>0</v>
-      </c>
-      <c r="F20" s="51" t="s">
+      <c r="E20" s="48">
+        <v>5</v>
+      </c>
+      <c r="F20" s="49" t="s">
         <v>29</v>
       </c>
-      <c r="G20" s="18">
-        <v>0</v>
+      <c r="G20" s="35">
+        <v>200</v>
       </c>
       <c r="H20" s="19">
         <f>E20*G20</f>
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="I20" s="20"/>
-      <c r="J20" s="51" t="s">
+      <c r="J20" s="49" t="s">
         <v>29</v>
       </c>
       <c r="K20" s="18"/>
@@ -1716,31 +1678,31 @@
       </c>
       <c r="M20" s="2"/>
     </row>
-    <row r="21" spans="1:13" ht="15.5">
+    <row r="21" spans="1:13" ht="15">
       <c r="A21" s="26" t="s">
         <v>19</v>
       </c>
       <c r="B21" s="14">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C21" s="35">
         <v>0</v>
       </c>
-      <c r="E21" s="50">
-        <v>0</v>
-      </c>
-      <c r="F21" s="51" t="s">
+      <c r="E21" s="48">
+        <v>1</v>
+      </c>
+      <c r="F21" s="49" t="s">
         <v>29</v>
       </c>
-      <c r="G21" s="18">
-        <v>0</v>
+      <c r="G21" s="35">
+        <v>800</v>
       </c>
       <c r="H21" s="19">
         <f>E21*G21</f>
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="I21" s="20"/>
-      <c r="J21" s="51" t="s">
+      <c r="J21" s="49" t="s">
         <v>29</v>
       </c>
       <c r="K21" s="18"/>
@@ -1750,18 +1712,18 @@
       </c>
       <c r="M21" s="2"/>
     </row>
-    <row r="22" spans="1:13" ht="15.5">
+    <row r="22" spans="1:13" ht="15">
       <c r="A22" s="26" t="s">
         <v>21</v>
       </c>
       <c r="B22" s="14">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C22" s="35">
         <v>0</v>
       </c>
-      <c r="E22" s="50"/>
-      <c r="F22" s="51" t="s">
+      <c r="E22" s="48"/>
+      <c r="F22" s="49" t="s">
         <v>29</v>
       </c>
       <c r="G22" s="18"/>
@@ -1770,7 +1732,7 @@
         <v>0</v>
       </c>
       <c r="I22" s="20"/>
-      <c r="J22" s="51" t="s">
+      <c r="J22" s="49" t="s">
         <v>29</v>
       </c>
       <c r="K22" s="18"/>
@@ -1780,15 +1742,15 @@
       </c>
       <c r="M22" s="2"/>
     </row>
-    <row r="23" spans="1:13" ht="15.5">
+    <row r="23" spans="1:13" ht="15">
       <c r="A23" s="26"/>
-      <c r="B23" s="47"/>
-      <c r="C23" s="52"/>
-      <c r="E23" s="50"/>
-      <c r="F23" s="51" t="s">
+      <c r="B23" s="45"/>
+      <c r="C23" s="50"/>
+      <c r="E23" s="48"/>
+      <c r="F23" s="49" t="s">
         <v>29</v>
       </c>
-      <c r="G23" s="18">
+      <c r="G23" s="35">
         <v>0</v>
       </c>
       <c r="H23" s="19">
@@ -1796,7 +1758,7 @@
         <v>0</v>
       </c>
       <c r="I23" s="20"/>
-      <c r="J23" s="51" t="s">
+      <c r="J23" s="49" t="s">
         <v>29</v>
       </c>
       <c r="K23" s="18"/>
@@ -1806,9 +1768,9 @@
       </c>
       <c r="M23" s="2"/>
     </row>
-    <row r="24" spans="1:13" ht="15.5">
-      <c r="A24" s="48"/>
-      <c r="B24" s="49" t="s">
+    <row r="24" spans="1:13" ht="15">
+      <c r="A24" s="46"/>
+      <c r="B24" s="47" t="s">
         <v>31</v>
       </c>
       <c r="C24" s="17">
@@ -1818,43 +1780,43 @@
       <c r="E24" s="26"/>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
-      <c r="H24" s="51"/>
+      <c r="H24" s="49"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
       <c r="L24" s="29"/>
       <c r="M24" s="2"/>
     </row>
-    <row r="25" spans="1:13" ht="15.5">
-      <c r="E25" s="48"/>
-      <c r="F25" s="49"/>
-      <c r="G25" s="49"/>
-      <c r="H25" s="58"/>
-      <c r="I25" s="49"/>
-      <c r="J25" s="49"/>
-      <c r="K25" s="59" t="s">
+    <row r="25" spans="1:13" ht="15">
+      <c r="E25" s="46"/>
+      <c r="F25" s="47"/>
+      <c r="G25" s="47"/>
+      <c r="H25" s="56"/>
+      <c r="I25" s="47"/>
+      <c r="J25" s="47"/>
+      <c r="K25" s="57" t="s">
         <v>52</v>
       </c>
       <c r="L25" s="17">
         <f>H19+H20+H21+H23+L19+L20+L21+L23+L22+H22</f>
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="M25" s="2"/>
     </row>
-    <row r="26" spans="1:13" ht="15.5">
+    <row r="26" spans="1:13" ht="15">
       <c r="M26" s="2"/>
     </row>
-    <row r="27" spans="1:13" ht="15.5">
+    <row r="27" spans="1:13" ht="15.6">
       <c r="A27" s="36" t="s">
         <v>32</v>
       </c>
-      <c r="B27" s="53"/>
-      <c r="C27" s="53"/>
-      <c r="D27" s="53"/>
+      <c r="B27" s="51"/>
+      <c r="C27" s="51"/>
+      <c r="D27" s="51"/>
       <c r="E27" s="12"/>
       <c r="M27" s="2"/>
     </row>
-    <row r="28" spans="1:13" ht="15.5">
+    <row r="28" spans="1:13" ht="15">
       <c r="A28" s="23" t="s">
         <v>33</v>
       </c>
@@ -1870,9 +1832,9 @@
       <c r="L28" s="2"/>
       <c r="M28" s="2"/>
     </row>
-    <row r="29" spans="1:13" ht="15.5">
-      <c r="A29" s="50"/>
-      <c r="B29" s="51" t="s">
+    <row r="29" spans="1:13" ht="15">
+      <c r="A29" s="48"/>
+      <c r="B29" s="49" t="s">
         <v>29</v>
       </c>
       <c r="C29" s="14"/>
@@ -1883,9 +1845,9 @@
       <c r="F29" s="2"/>
       <c r="M29" s="2"/>
     </row>
-    <row r="30" spans="1:13" ht="15.5">
-      <c r="A30" s="50"/>
-      <c r="B30" s="51" t="s">
+    <row r="30" spans="1:13" ht="15">
+      <c r="A30" s="48"/>
+      <c r="B30" s="49" t="s">
         <v>29</v>
       </c>
       <c r="C30" s="14"/>
@@ -1896,9 +1858,9 @@
       </c>
       <c r="F30" s="2"/>
     </row>
-    <row r="31" spans="1:13" ht="15.5">
-      <c r="A31" s="50"/>
-      <c r="B31" s="51" t="s">
+    <row r="31" spans="1:13" ht="15">
+      <c r="A31" s="48"/>
+      <c r="B31" s="49" t="s">
         <v>29</v>
       </c>
       <c r="C31" s="14"/>
@@ -1909,95 +1871,99 @@
       </c>
       <c r="F31" s="2"/>
     </row>
-    <row r="32" spans="1:13" ht="15.5">
-      <c r="A32" s="55"/>
-      <c r="B32" s="51" t="s">
+    <row r="32" spans="1:13" ht="15">
+      <c r="A32" s="53"/>
+      <c r="B32" s="49" t="s">
         <v>29</v>
       </c>
-      <c r="C32" s="47"/>
+      <c r="C32" s="45"/>
       <c r="D32" s="2"/>
-      <c r="E32" s="56">
+      <c r="E32" s="54">
         <f>A32*C32</f>
         <v>0</v>
       </c>
       <c r="F32" s="2"/>
     </row>
-    <row r="33" spans="1:15" ht="15.5">
-      <c r="A33" s="57"/>
-      <c r="B33" s="58"/>
-      <c r="C33" s="58" t="s">
+    <row r="33" spans="1:15" ht="15">
+      <c r="A33" s="55"/>
+      <c r="B33" s="56"/>
+      <c r="C33" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="D33" s="49"/>
+      <c r="D33" s="47"/>
       <c r="E33" s="19">
         <f>SUM(E29:E32)</f>
         <v>0</v>
       </c>
       <c r="F33" s="2"/>
     </row>
-    <row r="34" spans="1:15" ht="15.5">
+    <row r="34" spans="1:15" ht="15">
       <c r="F34" s="2"/>
     </row>
-    <row r="35" spans="1:15" ht="15.5">
+    <row r="35" spans="1:15" ht="15">
       <c r="F35" s="2"/>
     </row>
-    <row r="36" spans="1:15" ht="15.5">
-      <c r="A36" s="65" t="s">
-        <v>77</v>
-      </c>
-      <c r="B36" s="58"/>
-      <c r="C36" s="58"/>
-      <c r="D36" s="49"/>
-      <c r="E36" s="59"/>
+    <row r="36" spans="1:15" ht="15.6">
+      <c r="A36" s="63" t="s">
+        <v>76</v>
+      </c>
+      <c r="B36" s="56"/>
+      <c r="C36" s="56"/>
+      <c r="D36" s="47"/>
+      <c r="E36" s="57"/>
       <c r="F36" s="2"/>
     </row>
-    <row r="37" spans="1:15" ht="15.5">
-      <c r="A37" s="60"/>
-      <c r="B37" s="61"/>
-      <c r="C37" s="61"/>
+    <row r="37" spans="1:15" ht="15">
+      <c r="A37" s="58"/>
+      <c r="B37" s="59"/>
+      <c r="C37" s="59"/>
       <c r="D37" s="24"/>
       <c r="E37" s="25"/>
       <c r="F37" s="2"/>
     </row>
-    <row r="38" spans="1:15" ht="15.5">
-      <c r="A38" s="62" t="s">
+    <row r="38" spans="1:15" ht="15">
+      <c r="A38" s="60" t="s">
         <v>36</v>
       </c>
-      <c r="B38" s="13"/>
-      <c r="C38" s="51"/>
+      <c r="B38" s="13">
+        <v>500</v>
+      </c>
+      <c r="C38" s="49"/>
       <c r="D38" s="2"/>
       <c r="E38" s="27"/>
       <c r="F38" s="2"/>
       <c r="K38" s="2"/>
       <c r="L38" s="2"/>
     </row>
-    <row r="39" spans="1:15" ht="15.5">
-      <c r="A39" s="62" t="s">
+    <row r="39" spans="1:15" ht="15.6">
+      <c r="A39" s="60" t="s">
         <v>37</v>
       </c>
-      <c r="B39" s="13"/>
-      <c r="C39" s="51"/>
+      <c r="B39" s="13">
+        <v>100</v>
+      </c>
+      <c r="C39" s="49"/>
       <c r="D39" s="2"/>
       <c r="E39" s="27"/>
       <c r="F39" s="2"/>
       <c r="G39" s="8"/>
-      <c r="H39" s="74" t="s">
+      <c r="H39" s="72" t="s">
         <v>41</v>
       </c>
-      <c r="I39" s="74"/>
-      <c r="J39" s="74"/>
+      <c r="I39" s="72"/>
+      <c r="J39" s="72"/>
       <c r="K39" s="8"/>
       <c r="L39" s="8"/>
       <c r="M39" s="2"/>
     </row>
-    <row r="40" spans="1:15" ht="15.5">
+    <row r="40" spans="1:15" ht="15">
       <c r="A40" s="26"/>
-      <c r="B40" s="63"/>
+      <c r="B40" s="61"/>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
       <c r="E40" s="27"/>
       <c r="F40" s="2"/>
-      <c r="G40" s="72" t="s">
+      <c r="G40" s="70" t="s">
         <v>53</v>
       </c>
       <c r="H40" s="2" t="s">
@@ -2007,20 +1973,20 @@
       <c r="J40" s="2"/>
       <c r="L40" s="21">
         <f>B15</f>
-        <v>0</v>
+        <v>1933</v>
       </c>
       <c r="M40" s="32"/>
     </row>
-    <row r="41" spans="1:15" ht="15.5">
+    <row r="41" spans="1:15" ht="15">
       <c r="A41" s="30" t="s">
         <v>38</v>
       </c>
       <c r="B41" s="19"/>
       <c r="C41" s="7"/>
       <c r="D41" s="7"/>
-      <c r="E41" s="64"/>
+      <c r="E41" s="62"/>
       <c r="F41" s="2"/>
-      <c r="G41" s="72" t="s">
+      <c r="G41" s="70" t="s">
         <v>54</v>
       </c>
       <c r="H41" s="2" t="s">
@@ -2030,17 +1996,17 @@
       <c r="J41" s="2"/>
       <c r="L41" s="21">
         <f>+E14</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:15" ht="15.5">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" ht="15">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
       <c r="F42" s="2"/>
-      <c r="G42" s="72" t="s">
+      <c r="G42" s="70" t="s">
         <v>55</v>
       </c>
       <c r="H42" s="2" t="s">
@@ -2050,19 +2016,19 @@
       <c r="J42" s="2"/>
       <c r="L42" s="21">
         <f>+L15</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:15" ht="15.5">
-      <c r="A43" s="66" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" ht="15.6">
+      <c r="A43" s="64" t="s">
         <v>39</v>
       </c>
-      <c r="B43" s="67"/>
-      <c r="C43" s="67"/>
-      <c r="D43" s="49"/>
-      <c r="E43" s="59"/>
+      <c r="B43" s="65"/>
+      <c r="C43" s="65"/>
+      <c r="D43" s="47"/>
+      <c r="E43" s="57"/>
       <c r="F43" s="2"/>
-      <c r="G43" s="72" t="s">
+      <c r="G43" s="70" t="s">
         <v>56</v>
       </c>
       <c r="H43" s="2" t="s">
@@ -2075,7 +2041,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:15" ht="15.5">
+    <row r="44" spans="1:15" ht="15">
       <c r="A44" s="26" t="s">
         <v>40</v>
       </c>
@@ -2084,7 +2050,7 @@
       <c r="D44" s="2"/>
       <c r="E44" s="27"/>
       <c r="F44" s="2"/>
-      <c r="G44" s="72" t="s">
+      <c r="G44" s="70" t="s">
         <v>57</v>
       </c>
       <c r="H44" s="2" t="s">
@@ -2094,10 +2060,10 @@
       <c r="J44" s="2"/>
       <c r="L44" s="21">
         <f>+L25</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:15" ht="15.5">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" ht="15">
       <c r="A45" s="26" t="s">
         <v>42</v>
       </c>
@@ -2106,7 +2072,7 @@
       <c r="D45" s="2"/>
       <c r="E45" s="27"/>
       <c r="F45" s="2"/>
-      <c r="G45" s="72" t="s">
+      <c r="G45" s="70" t="s">
         <v>58</v>
       </c>
       <c r="H45" s="2" t="s">
@@ -2119,18 +2085,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:15" ht="15.5">
+    <row r="46" spans="1:15" ht="15">
       <c r="A46" s="26"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
       <c r="E46" s="27"/>
       <c r="F46" s="2"/>
-      <c r="G46" s="72" t="s">
+      <c r="G46" s="70" t="s">
         <v>64</v>
       </c>
-      <c r="H46" s="71" t="s">
-        <v>78</v>
+      <c r="H46" s="69" t="s">
+        <v>77</v>
       </c>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
@@ -2139,18 +2105,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:15" ht="15.5">
+    <row r="47" spans="1:15" ht="15">
       <c r="A47" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="B47" s="76">
-        <v>0</v>
+      <c r="B47" s="74">
+        <v>34</v>
       </c>
       <c r="C47" s="7"/>
       <c r="D47" s="7"/>
-      <c r="E47" s="64"/>
+      <c r="E47" s="62"/>
       <c r="F47" s="2"/>
-      <c r="G47" s="72"/>
+      <c r="G47" s="70"/>
       <c r="H47" s="2" t="s">
         <v>65</v>
       </c>
@@ -2159,14 +2125,14 @@
       <c r="L47" s="21"/>
       <c r="O47" s="2"/>
     </row>
-    <row r="48" spans="1:15" ht="15.5">
+    <row r="48" spans="1:15" ht="15">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
       <c r="E48" s="2"/>
       <c r="F48" s="2"/>
-      <c r="G48" s="72"/>
+      <c r="G48" s="70"/>
       <c r="H48" s="2" t="s">
         <v>45</v>
       </c>
@@ -2174,19 +2140,19 @@
       <c r="J48" s="2"/>
       <c r="L48" s="21">
         <f>SUM(L40:L47)</f>
-        <v>0</v>
+        <v>5770</v>
       </c>
       <c r="O48" s="2"/>
     </row>
-    <row r="49" spans="1:15" ht="15.5">
+    <row r="49" spans="1:15" ht="15">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
       <c r="E49" s="2"/>
       <c r="F49" s="2"/>
-      <c r="G49" s="72" t="s">
-        <v>74</v>
+      <c r="G49" s="70" t="s">
+        <v>73</v>
       </c>
       <c r="H49" s="2" t="s">
         <v>66</v>
@@ -2195,63 +2161,63 @@
       <c r="J49" s="2"/>
       <c r="L49" s="21">
         <f>+B47</f>
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="O49" s="2"/>
     </row>
-    <row r="50" spans="1:15" ht="15.5">
-      <c r="A50" s="66" t="s">
+    <row r="50" spans="1:15" ht="15.6">
+      <c r="A50" s="64" t="s">
         <v>44</v>
       </c>
-      <c r="B50" s="67"/>
-      <c r="C50" s="67"/>
-      <c r="D50" s="67"/>
-      <c r="E50" s="69"/>
+      <c r="B50" s="65"/>
+      <c r="C50" s="65"/>
+      <c r="D50" s="65"/>
+      <c r="E50" s="67"/>
       <c r="F50" s="2"/>
-      <c r="G50" s="73" t="s">
-        <v>73</v>
-      </c>
-      <c r="H50" s="71" t="s">
-        <v>81</v>
+      <c r="G50" s="71" t="s">
+        <v>72</v>
+      </c>
+      <c r="H50" s="69" t="s">
+        <v>80</v>
       </c>
       <c r="L50" s="21">
         <f>+E56</f>
-        <v>0</v>
+        <v>-4.1500000000000004</v>
       </c>
       <c r="O50" s="2"/>
     </row>
-    <row r="51" spans="1:15" ht="15.5">
+    <row r="51" spans="1:15" ht="15">
       <c r="A51" s="26" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
-      <c r="E51" s="13">
-        <v>0</v>
+      <c r="E51" s="35">
+        <v>-4.1500000000000004</v>
       </c>
       <c r="F51" s="2"/>
-      <c r="G51" s="72" t="s">
+      <c r="G51" s="70" t="s">
         <v>67</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
       <c r="L51" s="21">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="O51" s="2"/>
     </row>
-    <row r="52" spans="1:15" ht="15.5">
+    <row r="52" spans="1:15" ht="15">
       <c r="A52" s="26"/>
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
       <c r="E52" s="27"/>
       <c r="F52" s="2"/>
-      <c r="G52" s="72" t="s">
-        <v>69</v>
+      <c r="G52" s="70" t="s">
+        <v>68</v>
       </c>
       <c r="H52" s="2" t="s">
         <v>70</v>
@@ -2260,61 +2226,58 @@
       <c r="J52" s="2"/>
       <c r="L52" s="21">
         <f>L47+L48+L49+L50+L51</f>
-        <v>0</v>
+        <v>8799.85</v>
       </c>
       <c r="O52" s="2"/>
     </row>
-    <row r="53" spans="1:15" ht="15.5">
+    <row r="53" spans="1:15" ht="15">
       <c r="A53" s="26" t="s">
-        <v>80</v>
-      </c>
-      <c r="B53" s="68"/>
+        <v>79</v>
+      </c>
+      <c r="B53" s="66"/>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
       <c r="E53" s="13">
         <v>0</v>
       </c>
       <c r="F53" s="2"/>
-      <c r="G53" s="71"/>
+      <c r="G53" s="69"/>
       <c r="H53" s="2" t="s">
-        <v>71</v>
+        <v>47</v>
       </c>
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
       <c r="L53" s="21">
-        <v>0</v>
+        <v>9000</v>
       </c>
       <c r="O53" s="2"/>
     </row>
-    <row r="54" spans="1:15" ht="15.5">
+    <row r="54" spans="1:15" ht="15">
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
       <c r="E54" s="27"/>
       <c r="F54" s="2"/>
-      <c r="G54" s="71"/>
+      <c r="G54" s="69"/>
       <c r="H54" s="2" t="s">
-        <v>47</v>
+        <v>71</v>
       </c>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
       <c r="L54" s="21">
         <f>L53-L52</f>
-        <v>0</v>
+        <v>200.14999999999964</v>
       </c>
       <c r="O54" s="2"/>
     </row>
-    <row r="55" spans="1:15" ht="15.5">
+    <row r="55" spans="1:15" ht="15">
       <c r="A55" s="26"/>
-      <c r="B55" s="63"/>
+      <c r="B55" s="61"/>
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
       <c r="E55" s="27"/>
       <c r="F55" s="2"/>
-      <c r="G55" s="71"/>
-      <c r="H55" s="2" t="s">
-        <v>72</v>
-      </c>
+      <c r="G55" s="69"/>
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
       <c r="L55" s="21">
@@ -2322,25 +2285,25 @@
       </c>
       <c r="O55" s="2"/>
     </row>
-    <row r="56" spans="1:15" ht="15.5">
-      <c r="A56" s="48" t="s">
+    <row r="56" spans="1:15" ht="15">
+      <c r="A56" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="B56" s="70"/>
-      <c r="C56" s="49"/>
-      <c r="D56" s="59"/>
+      <c r="B56" s="68"/>
+      <c r="C56" s="47"/>
+      <c r="D56" s="57"/>
       <c r="E56" s="19">
         <f>E51+E53</f>
-        <v>0</v>
+        <v>-4.1500000000000004</v>
       </c>
       <c r="F56" s="2"/>
       <c r="O56" s="2"/>
     </row>
-    <row r="57" spans="1:15" ht="15.5">
+    <row r="57" spans="1:15" ht="15">
       <c r="F57" s="2"/>
       <c r="O57" s="2"/>
     </row>
-    <row r="58" spans="1:15" ht="15.5">
+    <row r="58" spans="1:15" ht="15">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
@@ -2349,7 +2312,7 @@
       <c r="F58" s="2"/>
       <c r="O58" s="2"/>
     </row>
-    <row r="59" spans="1:15" ht="15.5">
+    <row r="59" spans="1:15" ht="15">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
@@ -2364,9 +2327,9 @@
       <c r="L59" s="2"/>
       <c r="O59" s="2"/>
     </row>
-    <row r="60" spans="1:15" ht="15.5">
+    <row r="60" spans="1:15" ht="15.6">
       <c r="A60" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="8"/>
@@ -2381,7 +2344,7 @@
       <c r="L60" s="22"/>
       <c r="O60" s="2"/>
     </row>
-    <row r="61" spans="1:15" ht="15.5">
+    <row r="61" spans="1:15" ht="15">
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
@@ -2396,7 +2359,7 @@
       <c r="L61" s="2"/>
       <c r="M61" s="2"/>
     </row>
-    <row r="62" spans="1:15" ht="15.5">
+    <row r="62" spans="1:15" ht="15.6">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
@@ -2411,7 +2374,7 @@
       <c r="L62" s="2"/>
       <c r="M62" s="8"/>
     </row>
-    <row r="63" spans="1:15" ht="15.5">
+    <row r="63" spans="1:15" ht="15">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
@@ -2426,7 +2389,7 @@
       <c r="L63" s="2"/>
       <c r="M63" s="2"/>
     </row>
-    <row r="64" spans="1:15" ht="15.5">
+    <row r="64" spans="1:15" ht="15">
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
@@ -2441,7 +2404,7 @@
       <c r="L64" s="2"/>
       <c r="M64" s="2"/>
     </row>
-    <row r="65" spans="1:13" ht="15.5">
+    <row r="65" spans="1:13" ht="15">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
@@ -2456,7 +2419,7 @@
       <c r="L65" s="2"/>
       <c r="M65" s="2"/>
     </row>
-    <row r="66" spans="1:13" ht="15.5">
+    <row r="66" spans="1:13" ht="15.6">
       <c r="B66" s="2"/>
       <c r="C66" s="2"/>
       <c r="D66" s="2"/>
@@ -2470,11 +2433,11 @@
       <c r="L66" s="2"/>
       <c r="M66" s="2"/>
     </row>
-    <row r="67" spans="1:13" ht="15.5">
+    <row r="67" spans="1:13" ht="15">
       <c r="F67" s="2"/>
       <c r="M67" s="2"/>
     </row>
-    <row r="68" spans="1:13" ht="15.5">
+    <row r="68" spans="1:13" ht="15">
       <c r="F68" s="2"/>
       <c r="M68" s="2"/>
     </row>
@@ -2485,12 +2448,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -2499,7 +2456,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F1CDF4AE13F64D40BBB65824B29FAA7E" ma:contentTypeVersion="8" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0d2301f73a884384ddd5c8a4d00c99b5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="165b96c2-f4bb-42d4-bd0e-5bd22b3c2c99" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f44d8ff651ee59b55465c93f60004624" ns2:_="">
     <xsd:import namespace="165b96c2-f4bb-42d4-bd0e-5bd22b3c2c99"/>
@@ -2667,23 +2624,13 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B24100DD-9604-4D6D-B080-152095F3FAE0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="165b96c2-f4bb-42d4-bd0e-5bd22b3c2c99"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1677FD12-FF7E-4FED-B391-03DF70F45953}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -2691,7 +2638,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC46D7E8-5F30-4E91-A1E5-4030A3C193DF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2709,6 +2656,22 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B24100DD-9604-4D6D-B080-152095F3FAE0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="165b96c2-f4bb-42d4-bd0e-5bd22b3c2c99"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{cd62b7dd-4b48-44bd-90e7-e143a22c8ead}" enabled="0" method="" siteId="{cd62b7dd-4b48-44bd-90e7-e143a22c8ead}" removed="1"/>

</xml_diff>